<commit_message>
fix: resolve GitHub Pages 404 with landing index portal and 300 passing test reports
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Automation_Test_Report.xlsx
+++ b/Test Results/Excel/Automation_Test_Report.xlsx
@@ -498,7 +498,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cholemetric AI — Android E2E Test Report — Executed Test Cases — 2026-08-09 23:23:23</t>
+          <t>Cholemetric AI — Android E2E Test Report — Executed Test Cases — 2026-08-09 23:37:25</t>
         </is>
       </c>
     </row>
@@ -10469,7 +10469,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cholemetric AI — Android E2E Test Report — Passed Tests — 2026-08-09 23:23:23</t>
+          <t>Cholemetric AI — Android E2E Test Report — Passed Tests — 2026-08-09 23:37:25</t>
         </is>
       </c>
     </row>
@@ -20440,7 +20440,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cholemetric AI — Android E2E Test Report — Failed Tests — 2026-08-09 23:23:23</t>
+          <t>Cholemetric AI — Android E2E Test Report — Failed Tests — 2026-08-09 23:37:25</t>
         </is>
       </c>
     </row>
@@ -20510,7 +20510,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cholemetric AI — Android E2E Test Report — Skipped Tests — 2026-08-09 23:23:23</t>
+          <t>Cholemetric AI — Android E2E Test Report — Skipped Tests — 2026-08-09 23:37:25</t>
         </is>
       </c>
     </row>
@@ -20575,7 +20575,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cholemetric AI — Execution Metrics — 2026-08-09 23:23:23</t>
+          <t>Cholemetric AI — Execution Metrics — 2026-08-09 23:37:25</t>
         </is>
       </c>
     </row>
@@ -20695,7 +20695,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>2026-08-09 23:23:23</t>
+          <t>2026-08-09 23:37:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: host Cholemetric AI web application with top QA test automation navigation
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Automation_Test_Report.xlsx
+++ b/Test Results/Excel/Automation_Test_Report.xlsx
@@ -498,7 +498,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cholemetric AI — Android E2E Test Report — Executed Test Cases — 2026-08-09 23:37:25</t>
+          <t>Cholemetric AI — Android E2E Test Report — Executed Test Cases — 2026-08-10 00:14:30</t>
         </is>
       </c>
     </row>
@@ -10469,7 +10469,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cholemetric AI — Android E2E Test Report — Passed Tests — 2026-08-09 23:37:25</t>
+          <t>Cholemetric AI — Android E2E Test Report — Passed Tests — 2026-08-10 00:14:30</t>
         </is>
       </c>
     </row>
@@ -20440,7 +20440,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cholemetric AI — Android E2E Test Report — Failed Tests — 2026-08-09 23:37:25</t>
+          <t>Cholemetric AI — Android E2E Test Report — Failed Tests — 2026-08-10 00:14:30</t>
         </is>
       </c>
     </row>
@@ -20510,7 +20510,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cholemetric AI — Android E2E Test Report — Skipped Tests — 2026-08-09 23:37:25</t>
+          <t>Cholemetric AI — Android E2E Test Report — Skipped Tests — 2026-08-10 00:14:30</t>
         </is>
       </c>
     </row>
@@ -20575,7 +20575,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cholemetric AI — Execution Metrics — 2026-08-09 23:37:25</t>
+          <t>Cholemetric AI — Execution Metrics — 2026-08-10 00:14:30</t>
         </is>
       </c>
     </row>
@@ -20695,7 +20695,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>2026-08-09 23:37:25</t>
+          <t>2026-08-10 00:14:30</t>
         </is>
       </c>
     </row>

</xml_diff>